<commit_message>
HU-036: PRU sem objeto custom — Decision Matrix (BRE) como tabela de referencia
T09/T10/T15 e abas de decisoes/arquitetura ajustadas: o PRU vive numa
Decision Matrix versionada (entradas Pais/Marca/Modelo/Ano, saida
ValorReferencia), carga por CSV nativo, qualquer marca sem depender de
Product2; Flow/Expression Set busca o valor e grava no
AppraisalItemProviderVal, que o valuador confirma.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/hu036-avaluo/HU036_Tarefas_Tecnicas.xlsx
+++ b/deploy/hu036-avaluo/HU036_Tarefas_Tecnicas.xlsx
@@ -504,27 +504,27 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Objeto/tabela mestre do PRU por país</t>
+          <t xml:space="preserve">Decision Matrix do PRU por país (BRE)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRU (custom até OEM)</t>
+          <t xml:space="preserve">Decision Matrix (Lookup Tables / BRE)</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metadata</t>
+          <t xml:space="preserve">Config (BRE)</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom</t>
+          <t xml:space="preserve">Nativo (licenciado)</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blue book / valor de referência com dimensão por país (GQ-CA-01-157). Carga massiva/unitária.</t>
+          <t xml:space="preserve">Blue book / valor de referência SEM objeto custom: Decision Matrix com entradas País, Marca, Modelo, Año (+Versión) e saída ValorReferencia. Versionada (revisão trimestral/mensal = nova versão); cobre qualquer marca, sem depender de Product2. GQ-CA-01-157.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -551,7 +551,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Loader</t>
+          <t xml:space="preserve">CSV da Decision Matrix</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -561,12 +561,12 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom</t>
+          <t xml:space="preserve">Nativo (licenciado)</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Popular a tabela mestre do PRU; atualização periódica (trimestral c/ revisão mensal).</t>
+          <t xml:space="preserve">Carga inicial via CSV nativo da Decision Matrix; cada atualização trimestral/mensal é uma nova versão da matriz (auditável).</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registrar valor de referência do avalúo apontando para a tabela mestre do PRU.</t>
+          <t xml:space="preserve">Flow/Expression Set busca na Decision Matrix (País+Marca+Modelo+Año do AppraisalItem) e grava o valor sugerido no AppraisalItemProviderVal; o valuador confirma. Provider = Account do provedor (PRU).</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -1183,17 +1183,17 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tabela mestre por país; ProviderVal referencia.</t>
+          <t xml:space="preserve">Decision Matrix (BRE) por país — SEM objeto custom; ProviderVal recebe o valor via Flow.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom</t>
+          <t xml:space="preserve">Nativo (BRE)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom até integração OEM.</t>
+          <t xml:space="preserve">Nativo licenciado (BRE); versões = auditoria das atualizações.</t>
         </is>
       </c>
     </row>
@@ -1573,17 +1573,17 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRU (custom)</t>
+          <t xml:space="preserve">PRU (Decision Matrix / BRE)</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dado mestre de referência por país.</t>
+          <t xml:space="preserve">Tabela de referência por país no BRE, versionada; carga por CSV.</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referenciado por AppraisalItemProviderVal.</t>
+          <t xml:space="preserve">Consultada por Flow/Expression Set; o valor gravado vive em AppraisalItemProviderVal.</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4. AppraisalItemProviderVal: valor de referência do PRU (por país).</t>
+          <t xml:space="preserve">4. AppraisalItemProviderVal: valor de referência buscado na Decision Matrix do PRU (por país) via Flow.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HU-036: confirmacoes do Object Reference oficial do Appraisal
FinalAppraisalValue/TotalItemFinalValue/TotalAdjustmentValue calculados
(confirmado); ReferenceRecordId = Account/Case/Lead/Opportunity; PurposeType
restrito Sale/Trade-In; AppraisedById User/Contact (ancora do valuador
externo); Status nao restrito (estados do fluxo); ValidityEndDate e
AppraisalHistory nativos; T01 = habilitar Appraisal Management. PRU:
versionamento por vigencia+rank das Decision Matrices confirmado no doc.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/hu036-avaluo/HU036_Tarefas_Tecnicas.xlsx
+++ b/deploy/hu036-avaluo/HU036_Tarefas_Tecnicas.xlsx
@@ -188,7 +188,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verificar se a família Appraisal está ativa na org (Automotive Cloud).</t>
+          <t xml:space="preserve">Habilitar Automotive + Appraisal Management (regra oficial de acesso do objeto Appraisal, API v63+).</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -230,7 +230,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Travar API names reais e confirmar se FinalAppraisalValue é FORMULA. Base para o build.</t>
+          <t xml:space="preserve">CONFIRMADO no Object Reference: FinalAppraisalValue, TotalItemFinalValue e TotalAdjustmentValue sao CALCULADOS (valuador nao digita). Describe agora foca AppraisalItem e AppraisalItemProviderVal (campos ainda nao confirmados).</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERD: parent = UM entre Opportunity/Account/Lead/Case/Financial Account. GrupoQ: Opportunity ou Account. + Contact e User.</t>
+          <t xml:space="preserve">OFICIAL (Object Reference): ReferenceRecordId polimórfico = Account, Case, Lead ou Opportunity. GrupoQ: Opportunity. PurposeType = Trade-In (picklist restrito). AppraisedById = User (valuador interno) ou Contact (externo).</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1205,17 +1205,17 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Calculado nativamente; valuador não digita.</t>
+          <t xml:space="preserve">CONFIRMADO no Object Reference: campo calculado (TotalItemFinalValue + TotalAdjustmentValue).</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nativo (a confirmar)</t>
+          <t xml:space="preserve">Nativo (CONFIRMADO)</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirmar no describe se é FORMULA/rollup.</t>
+          <t xml:space="preserve">Doc oficial do objeto Appraisal (API v63+).</t>
         </is>
       </c>
     </row>
@@ -1227,7 +1227,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lookup polimórfico: UM entre Opportunity, Account, Lead, Case ou Financial Account (+ Contact, User).</t>
+          <t xml:space="preserve">ReferenceRecordId polimórfico: Account, Case, Lead ou Opportunity (oficial). AppraisedById: Contact ou User. InitiatedById: Account/Contact/User.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONFIRMADO no ERD oficial.</t>
+          <t xml:space="preserve">CONFIRMADO no Object Reference oficial. Bonus nativo: ValidityEndDate (vigencia do avaluo) e AppraisalHistory (rastreio de campos).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HU-036: runbook con deploy DEV confirmado y columna Status en la planilla T01-T21
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/hu036-avaluo/HU036_Tarefas_Tecnicas.xlsx
+++ b/deploy/hu036-avaluo/HU036_Tarefas_Tecnicas.xlsx
@@ -106,6 +106,7 @@
     <col min="6" max="6" width="52" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="8" customWidth="1"/>
+    <col min="9" max="9" width="44" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -159,6 +160,11 @@
           <t xml:space="preserve">Est. (d)</t>
         </is>
       </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status (23/07)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -201,6 +207,11 @@
           <t xml:space="preserve">0.5</t>
         </is>
       </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONCLUIDA 23/07 - feature verificada (describe: familia createable)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -243,6 +254,11 @@
           <t xml:space="preserve">0.5</t>
         </is>
       </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONCLUIDA 23/07 - describe + Object Reference oficiais</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -285,6 +301,11 @@
           <t xml:space="preserve">1</t>
         </is>
       </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONCLUIDA 23/07 - desplegado via paquete v2 (4 campos + Permission Set)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -327,6 +348,11 @@
           <t xml:space="preserve">0.5</t>
         </is>
       </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONCLUIDA 23/07 - Work Type Avaluo criado</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -369,6 +395,11 @@
           <t xml:space="preserve">1</t>
         </is>
       </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONCLUIDA 23/07 - reuso do territory da sucursal (rename pendente)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -411,6 +442,11 @@
           <t xml:space="preserve">1</t>
         </is>
       </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARCIAL - recurso de teste ativo; valuadores reais = insumo GrupoQ</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -453,6 +489,11 @@
           <t xml:space="preserve">1</t>
         </is>
       </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendente - modelagem pronta; aguarda proveedor real (insumo)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -495,6 +536,11 @@
           <t xml:space="preserve">1</t>
         </is>
       </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proximo bloco (Flow 2)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -537,6 +583,11 @@
           <t xml:space="preserve">2</t>
         </is>
       </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EM CURSO - matriz provisoria; estrutura final depende do insumo PRU</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -579,6 +630,11 @@
           <t xml:space="preserve">1</t>
         </is>
       </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aguarda insumo GrupoQ (arquivo PRU)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -621,6 +677,11 @@
           <t xml:space="preserve">2</t>
         </is>
       </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendente</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -663,6 +724,11 @@
           <t xml:space="preserve">0.5</t>
         </is>
       </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendente</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -705,6 +771,11 @@
           <t xml:space="preserve">0.5</t>
         </is>
       </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONCLUIDA 23/07 - decisao registrada: Opportunity + Trade-In</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -747,6 +818,11 @@
           <t xml:space="preserve">1</t>
         </is>
       </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendente - teste na UI</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -789,6 +865,11 @@
           <t xml:space="preserve">0.5</t>
         </is>
       </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proximo bloco (Flow 1: matriz -&gt; ProviderVal + InitialValue)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -831,6 +912,11 @@
           <t xml:space="preserve">0.5</t>
         </is>
       </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendente</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -873,6 +959,11 @@
           <t xml:space="preserve">1.5</t>
         </is>
       </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proximo bloco (Flow 3: cierre -&gt; Opportunity)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -915,6 +1006,11 @@
           <t xml:space="preserve">0.5</t>
         </is>
       </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proximo bloco (Flow 3)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -957,6 +1053,11 @@
           <t xml:space="preserve">0.5</t>
         </is>
       </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendente</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -999,6 +1100,11 @@
           <t xml:space="preserve">0.5</t>
         </is>
       </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendente</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1039,6 +1145,11 @@
       <c r="H24" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendente - depende de T01-T20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HU-036: deploy v4 success en DEV - runbook y T01-T21 actualizados
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/hu036-avaluo/HU036_Tarefas_Tecnicas.xlsx
+++ b/deploy/hu036-avaluo/HU036_Tarefas_Tecnicas.xlsx
@@ -303,7 +303,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONCLUIDA 23/07 - desplegado via paquete v2 (4 campos + Permission Set)</t>
+          <t xml:space="preserve">CONCLUIDA 23/07 - paquete v4 (campos en ingles por naming GRPQM + Permission Set AppraisalManagement)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EM CURSO - matriz provisoria; estrutura final depende do insumo PRU</t>
+          <t xml:space="preserve">CONCLUIDA em DEV 23/07 - matriz ativa (V1); estrutura final depende do insumo PRU</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aguarda insumo GrupoQ (arquivo PRU)</t>
+          <t xml:space="preserve">Carga de teste feita (12 filas, 23/07); carga REAL aguarda insumo GrupoQ</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proximo bloco (Flow 1: matriz -&gt; ProviderVal + InitialValue)</t>
+          <t xml:space="preserve">Flow desplegado em Draft 23/07 (Appraisal Item After Handler) - ativar + teste</t>
         </is>
       </c>
     </row>

</xml_diff>